<commit_message>
Rename UPB Eventos.xlsx → Eventos.xlsx · skip section/header rows
- Filename ahora es Eventos.xlsx (no UPB Eventos.xlsx).
- extract_events salta filas-cabecera ("#", "Interprete") y filas-
  separador ("BANDA"/"ACÚSTICAS") dentro de cada hoja de evento, así un
  evento puede tener su lista completa con secciones (como Muela = todo
  el repertorio en banda + acústicas).
- extract_songs: la hoja "Unirock" ahora es opcional en el repertorio
  xlsx (migró completamente a Eventos.xlsx).
- Streamlit: 4to uploader pide "Eventos.xlsx".
- Subo Eventos.xlsx (Unirock × 9 + Muela × 39 songs) y Repertorio
  actualizado (sin la hoja Unirock).
</commit_message>
<xml_diff>
--- a/UPB Repertorio 2026 DEF.xlsx
+++ b/UPB Repertorio 2026 DEF.xlsx
@@ -5,19 +5,18 @@
   <fileSharing readOnlyRecommended="0" userName="luigi"/>
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="1" xWindow="240" yWindow="60" windowWidth="0" windowHeight="0" tabRatio="500"/>
+    <workbookView activeTab="0" xWindow="240" yWindow="60" windowWidth="0" windowHeight="0" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Repertorio" sheetId="1" r:id="rId4"/>
-    <sheet name="Unirock" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1779282532" val="1234" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1779282532" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="selection"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1779282532" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1779282532"/>
+      <pm:revision xmlns:pm="smNativeData" day="1779288039" val="1234" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1779288039" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="selection"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1779288039" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1779288039"/>
       <pm:pdfExportOpt xmlns:pm="smNativeData" pagesRangeIndex="1" pagesSelectionIndex="0" qualityIndex="2" embedFonts="2" useJpegs="0" useSubsetFonts="1" useAlpha="1" relativeLinks="0" taggedPdf="1" pane="0" zoom="0" zoomScale="100" layout="0" includeDoc="0" viewFlags="0" openViewer="1" jpegQuality="90" flags="252" exportWsNames="1" dpi="2" resample="1" name="C:\Users\luigi\OneDrive\Escritorio\UPB\2026\UPB Repertorio 2026  def.pdf"/>
     </ext>
   </extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="127">
   <si>
     <t>BANDA</t>
   </si>
@@ -419,57 +418,6 @@
   </si>
   <si>
     <t>Golden Hour</t>
-  </si>
-  <si>
-    <t>Unirock</t>
-  </si>
-  <si>
-    <t>Duración</t>
-  </si>
-  <si>
-    <t>Mayo</t>
-  </si>
-  <si>
-    <t>Junio</t>
-  </si>
-  <si>
-    <t>lunes</t>
-  </si>
-  <si>
-    <t>martes</t>
-  </si>
-  <si>
-    <t>miércoles</t>
-  </si>
-  <si>
-    <t>jueves</t>
-  </si>
-  <si>
-    <t>viernes</t>
-  </si>
-  <si>
-    <t>sábado</t>
-  </si>
-  <si>
-    <t>domingo</t>
-  </si>
-  <si>
-    <t>San Agustín</t>
-  </si>
-  <si>
-    <t>Ensayo</t>
-  </si>
-  <si>
-    <t>UniRock</t>
-  </si>
-  <si>
-    <t>Tiquipaya</t>
-  </si>
-  <si>
-    <t>Anglo</t>
-  </si>
-  <si>
-    <t>Open Campus</t>
   </si>
 </sst>
 </file>
@@ -490,7 +438,7 @@
     <numFmt numFmtId="20" formatCode="h:mm"/>
     <numFmt numFmtId="165" formatCode="[h]:mm;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -498,7 +446,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779282532" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779288039" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -513,7 +461,7 @@
       <sz val="8"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779282532" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779288039" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="160" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -528,7 +476,7 @@
       <sz val="8"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779282532" fgClr="FFFF00" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1779288039" fgClr="FFFF00" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="160" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -536,55 +484,8 @@
         </ext>
       </extLst>
     </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="8"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779282532" ulstyle="none" kern="1">
-            <pm:latin face="Arial" sz="160" lang="default"/>
-            <pm:cs face="Times New Roman" sz="360" lang="default"/>
-            <pm:ea face="SimSun" sz="360" lang="default"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b/>
-      <color rgb="FF000000"/>
-      <sz val="8"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779282532" ulstyle="none" kern="1">
-            <pm:latin face="Arial" sz="160" lang="default" weight="bold"/>
-            <pm:cs face="Times New Roman" sz="200" lang="default" weight="bold"/>
-            <pm:ea face="SimSun" sz="200" lang="default" weight="bold"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1779282532" ulstyle="none" kern="1">
-            <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
-            <pm:cs face="Times New Roman" sz="200" lang="default"/>
-            <pm:ea face="SimSun" sz="200" lang="default"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -600,7 +501,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="00FF0000" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="100" fgClr="00FF0000" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -611,7 +512,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -622,7 +523,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="76" fgClr="0000FFFF" bgLvl="24" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="76" fgClr="0000FFFF" bgLvl="24" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -633,7 +534,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -644,7 +545,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -655,7 +556,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="00FFFF00" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="100" fgClr="00FFFF00" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -666,7 +567,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="75" fgClr="0000FF00" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="75" fgClr="0000FF00" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -677,7 +578,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="75" fgClr="0000FFFF" bgLvl="100" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="75" fgClr="0000FFFF" bgLvl="100" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -688,7 +589,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="64" fgClr="00FF00FF" bgLvl="36" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="64" fgClr="00FF00FF" bgLvl="36" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -699,24 +600,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00FFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1779282532" type="1" fgLvl="100" fgClr="0000FFFF" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1779288039" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -732,7 +622,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532"/>
+          <pm:border xmlns:pm="smNativeData" id="1779288039"/>
         </ext>
       </extLst>
     </border>
@@ -751,7 +641,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -775,7 +665,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -799,7 +689,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -823,7 +713,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -847,7 +737,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -870,7 +760,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -893,7 +783,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -917,7 +807,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -941,7 +831,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -965,7 +855,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532">
+          <pm:border xmlns:pm="smNativeData" id="1779288039">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -989,26 +879,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1779282532"/>
+          <pm:border xmlns:pm="smNativeData" id="1779288039"/>
         </ext>
       </extLst>
     </border>
@@ -1016,7 +887,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1051,48 +922,6 @@
     <xf numFmtId="1" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -1100,10 +929,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1779282532" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1779288039" count="1">
         <pm:charStyle name="Normal" fontId="0"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1779282532" count="18">
+      <pm:colors xmlns:pm="smNativeData" id="1779288039" count="18">
         <pm:color name="Color 24" rgb="FFFF9E"/>
         <pm:color name="Color 25" rgb="9EFF9E"/>
         <pm:color name="Color 26" rgb="A3A300"/>
@@ -3782,7 +3611,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779282532" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1779288039" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3791,1188 +3620,17 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779282532" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779282532" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1779282532" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1779282532" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1779288039" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1779288039" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1779288039" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1779288039" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779282532" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
-        <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
-        <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
-      </pm:sheetPrefs>
-    </ext>
-  </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:AD29"/>
-  <sheetFormatPr baseColWidth="9" defaultColWidth="10.000000" defaultRowHeight="13.45"/>
-  <cols>
-    <col min="1" max="1" width="2.414414" customWidth="1"/>
-    <col min="2" max="2" width="13.306306" customWidth="1"/>
-    <col min="3" max="3" width="23.954955" customWidth="1"/>
-    <col min="4" max="4" width="6.981982" customWidth="1"/>
-    <col min="5" max="5" width="6.414414" customWidth="1"/>
-    <col min="6" max="6" width="8.423423" customWidth="1"/>
-    <col min="7" max="7" width="10.099099" customWidth="1"/>
-    <col min="8" max="8" width="6.738739" customWidth="1"/>
-    <col min="9" max="9" width="3.216216" customWidth="1"/>
-    <col min="10" max="10" width="7.207207" customWidth="1"/>
-    <col min="11" max="11" width="6.414414" customWidth="1"/>
-    <col min="12" max="12" width="8.108108" customWidth="1"/>
-    <col min="13" max="13" width="6.414414" customWidth="1"/>
-    <col min="14" max="14" width="6.810811" customWidth="1"/>
-    <col min="15" max="15" width="6.414414" customWidth="1"/>
-    <col min="16" max="16" width="6.738739" customWidth="1"/>
-    <col min="17" max="17" width="6.414414" customWidth="1"/>
-    <col min="18" max="18" width="5.783784" customWidth="1"/>
-    <col min="19" max="19" width="2.090090" customWidth="1"/>
-    <col min="20" max="20" width="6.900901" customWidth="1"/>
-    <col min="21" max="21" width="2.090090" customWidth="1"/>
-    <col min="22" max="22" width="4.396396" customWidth="1"/>
-    <col min="23" max="23" width="3.216216" customWidth="1"/>
-    <col min="24" max="24" width="5.450450" customWidth="1"/>
-    <col min="25" max="25" width="2.414414" customWidth="1"/>
-    <col min="26" max="26" width="2.567568" customWidth="1"/>
-    <col min="27" max="27" width="8.657658" customWidth="1"/>
-    <col min="28" max="28" width="5.315315" customWidth="1"/>
-    <col min="29" max="29" width="4.315315" customWidth="1"/>
-    <col min="30" max="31" width="6.414414" customWidth="1"/>
-    <col min="32" max="32" width="10.099099" customWidth="1"/>
-    <col min="33" max="33" width="6.414414" customWidth="1"/>
-    <col min="36" max="37" width="6.414414" customWidth="1"/>
-    <col min="38" max="38" width="6.981982" customWidth="1"/>
-    <col min="39" max="42" width="6.414414" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:25">
-      <c r="A1" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
-    </row>
-    <row r="2" spans="1:27">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27">
-      <c r="A3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y3" s="4">
-        <f>(E3+G3+I3+K3+M3+O3+Q3+S3+U3+W3)/D3</f>
-        <v>52</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28">
-      <c r="A4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="X4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y4" s="10">
-        <f>(E4+G4+I4+K4+M4+O4+Q4+S4+U4+W4)/D4</f>
-        <v>52.5</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28">
-      <c r="A5" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="X5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y5" s="10">
-        <f>(E5+G5+I5+K5+M5+O5+Q5+S5+U5+W5)/D5</f>
-        <v>55</v>
-      </c>
-      <c r="AA5" s="27" t="n">
-        <v>0.139583333333333348</v>
-      </c>
-      <c r="AB5" s="28" t="n">
-        <v>0.770833333333333393</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28">
-      <c r="A6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="X6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y6" s="10">
-        <f>(E6+G6+I6+K6+M6+O6+Q6+S6+U6+W6)/D6</f>
-        <v>32</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB6" s="28" t="n">
-        <v>0.854166666666666607</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="2" customFormat="1" ht="11.15">
-      <c r="A7" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="X7" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y7" s="10">
-        <f>(E7+G7+I7+K7+M7+O7+Q7+S7+U7+W7)/D7</f>
-        <v>46</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB7" s="29" t="n">
-        <v>1.0625</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28">
-      <c r="A8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
-      <c r="V8" s="4"/>
-      <c r="W8" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="X8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y8" s="10">
-        <f>(E8+G8+I8+K8+M8+O8+Q8+S8+U8+W8)/D8</f>
-        <v>48</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>4</v>
-      </c>
-      <c r="AB8" s="30" t="n">
-        <v>1.22916666666666674</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28">
-      <c r="A9" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="X9" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y9" s="10">
-        <f>(E9+G9+I9+K9+M9+O9+Q9+S9+U9+W9)/D9</f>
-        <v>66.6666666666666714</v>
-      </c>
-      <c r="AA9" s="27" t="n">
-        <v>0.354166666666666696</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30">
-      <c r="A10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>71</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="X10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y10" s="10">
-        <f>(E10+G10+I10+K10+M10+O10+Q10+S10+U10+W10)/D10</f>
-        <v>68.2000000000000028</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB10" s="31" t="n">
-        <v>58</v>
-      </c>
-      <c r="AC10" s="27"/>
-      <c r="AD10" s="27"/>
-    </row>
-    <row r="11" spans="1:28">
-      <c r="A11" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y11" s="10">
-        <f>(E11+G11+I11+K11+M11+O11+Q11+S11+U11+W11)/D11</f>
-        <v>47.5</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>4</v>
-      </c>
-      <c r="AB11" s="30" t="n">
-        <v>0.0430555555555555536</v>
-      </c>
-    </row>
-    <row r="13" spans="2:16">
-      <c r="B13" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-    </row>
-    <row r="14" spans="2:16">
-      <c r="B14" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="I14" s="13"/>
-      <c r="J14" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="K14" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="L14" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="M14" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="N14" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="O14" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="P14" s="14" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="15" spans="2:16">
-      <c r="B15" s="15" t="n">
-        <v>46146</v>
-      </c>
-      <c r="C15" s="15" t="n">
-        <v>46147</v>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>46148</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>46149</v>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>46150</v>
-      </c>
-      <c r="G15" s="15" t="n">
-        <v>46151</v>
-      </c>
-      <c r="H15" s="15" t="n">
-        <v>46152</v>
-      </c>
-      <c r="I15" s="13"/>
-      <c r="J15" s="15" t="n">
-        <v>46174</v>
-      </c>
-      <c r="K15" s="15" t="n">
-        <v>46175</v>
-      </c>
-      <c r="L15" s="15" t="n">
-        <v>46176</v>
-      </c>
-      <c r="M15" s="15" t="n">
-        <v>46177</v>
-      </c>
-      <c r="N15" s="15" t="n">
-        <v>46178</v>
-      </c>
-      <c r="O15" s="15" t="n">
-        <v>46179</v>
-      </c>
-      <c r="P15" s="15" t="n">
-        <v>46180</v>
-      </c>
-    </row>
-    <row r="16" spans="2:16">
-      <c r="B16" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="H16" s="15"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="L16" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="P16" s="15"/>
-    </row>
-    <row r="17" spans="2:16">
-      <c r="B17" s="1"/>
-      <c r="C17" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="D17" s="14"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="24"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="20"/>
-      <c r="P17" s="14"/>
-    </row>
-    <row r="18" spans="2:10">
-      <c r="B18" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-    </row>
-    <row r="19" spans="2:10">
-      <c r="B19" s="15" t="n">
-        <v>46153</v>
-      </c>
-      <c r="C19" s="15" t="n">
-        <v>46154</v>
-      </c>
-      <c r="D19" s="15" t="n">
-        <v>46155</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <v>46156</v>
-      </c>
-      <c r="F19" s="15" t="n">
-        <v>46157</v>
-      </c>
-      <c r="G19" s="15" t="n">
-        <v>46158</v>
-      </c>
-      <c r="H19" s="15" t="n">
-        <v>46159</v>
-      </c>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-    </row>
-    <row r="20" spans="2:10">
-      <c r="B20" s="15"/>
-      <c r="C20" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="G20" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="H20" s="15"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
-    </row>
-    <row r="21" spans="2:10">
-      <c r="B21" s="14"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-    </row>
-    <row r="22" spans="2:10">
-      <c r="B22" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-    </row>
-    <row r="23" spans="2:10">
-      <c r="B23" s="15" t="n">
-        <v>46160</v>
-      </c>
-      <c r="C23" s="15" t="n">
-        <v>46161</v>
-      </c>
-      <c r="D23" s="15" t="n">
-        <v>46162</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>46163</v>
-      </c>
-      <c r="F23" s="15" t="n">
-        <v>46164</v>
-      </c>
-      <c r="G23" s="15" t="n">
-        <v>46165</v>
-      </c>
-      <c r="H23" s="15" t="n">
-        <v>46166</v>
-      </c>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-    </row>
-    <row r="24" spans="2:10">
-      <c r="B24" s="15"/>
-      <c r="C24" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="H24" s="15"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
-    </row>
-    <row r="25" spans="2:10">
-      <c r="B25" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
-    </row>
-    <row r="26" spans="2:10">
-      <c r="B26" s="15" t="n">
-        <v>46167</v>
-      </c>
-      <c r="C26" s="15" t="n">
-        <v>46168</v>
-      </c>
-      <c r="D26" s="15" t="n">
-        <v>46169</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>46170</v>
-      </c>
-      <c r="F26" s="15" t="n">
-        <v>46171</v>
-      </c>
-      <c r="G26" s="15" t="n">
-        <v>46172</v>
-      </c>
-      <c r="H26" s="15" t="n">
-        <v>46173</v>
-      </c>
-      <c r="I26" s="13"/>
-      <c r="J26" s="13"/>
-    </row>
-    <row r="27" spans="2:10">
-      <c r="B27" s="15"/>
-      <c r="C27" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="D27" s="15"/>
-      <c r="E27" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="F27" s="15"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
-    </row>
-    <row r="28" spans="2:10">
-      <c r="B28" s="14"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="H28" s="14"/>
-      <c r="I28" s="13"/>
-      <c r="J28" s="13"/>
-    </row>
-    <row r="29" spans="2:10">
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
-      <c r="J29" s="13"/>
-    </row>
-  </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="J13:P13"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="N16:N17"/>
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="P16:P17"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="H27:H28"/>
-  </mergeCells>
-  <printOptions>
-    <extLst>
-      <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1779282532" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
-      </ext>
-    </extLst>
-  </printOptions>
-  <pageMargins left="0.787500" right="0.787500" top="0.787500" bottom="0.787500" header="0.393750" footer="0.393750"/>
-  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="1" pageOrder="overThenDown"/>
-  <headerFooter>
-    <extLst>
-      <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1779282532" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1779282532" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1779282532" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1779282532" Id="1" type="0" value="0"/>
-      </ext>
-    </extLst>
-  </headerFooter>
-  <extLst>
-    <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779282532" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1779288039" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>